<commit_message>
fix: AttributionTextNormalizer was not using the right delimiter for `remove_sentences_starting_with`
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution_par_mot.xlsx
+++ b/tests/integration/test_data/test_attribution_par_mot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BEB1EC-26AC-4141-ACBF-E1CDDCFBE3FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEE86BA-1668-5848-ACCE-3498FEEC95F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34400" yWindow="500" windowWidth="34400" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mots clés" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="46">
   <si>
     <t>Lecture</t>
   </si>
@@ -193,18 +193,12 @@
     <t>Fake</t>
   </si>
   <si>
-    <t>Madam Fake</t>
-  </si>
-  <si>
     <t xml:space="preserve">L’article L. 162‑1‑19 du code de la sécurité sociale est complété par un alinéa ainsi rédigé :
   « La communication prévue au premier alinéa concerne notamment les informations portant sur des faits à caractère frauduleux commis par un professionnel de santé. »
 I. – La perte de recettes pour l’État est compensée à due concurrence par la création d’une taxe additionnelle à l’accise sur les tabacs prévue au chapitre IV du titre Ier du livre III du code des impositions sur les biens et services.
 II. – La perte de recettes pour l’État est compensée à due concurrence par la création d’une taxe additionnelle à l’accise sur les tabacs prévue au chapitre IV du titre Ier du livre III du code des impositions sur les biens et services.
 « III. – Le montant mentionné aux I et II est cumulable avec les autres dispositifs d’exonérations de cotisations patronales de sécurité sociale dans la limite des cotisations patronales de sécurité sociale, ainsi que des contributions patronales recouvrées suivant les mêmes règles, restant dues par l’employeur, et, pour le reliquat éventuel, dans la limite des cotisations salariales de sécurité sociale précomptées, au titre de l’ensemble de la rémunération du salarié concerné.
 </t>
-  </si>
-  <si>
-    <t>Fake,Fake</t>
   </si>
   <si>
     <t>I. – À la fin du I de l’article 999 du code général des impôts, les mots : « et dans une limite annuelle égale à 7 500 € » sont supprimés.
@@ -239,12 +233,12 @@
     <t>Num amdt</t>
   </si>
   <si>
-    <t>Madam Fake,Mister Fake</t>
-  </si>
-  <si>
     <t>Le code du travail est ainsi modifié :
 1° L’article L. 5132-17 est ainsi rétabli :
 « Art. L. 5132-17 – Les usagers du système de santé bénéficient de la permanence des soins dans les conditions prévues par le présent code.</t>
+  </si>
+  <si>
+    <t>Mister Fake</t>
   </si>
 </sst>
 </file>
@@ -565,7 +559,7 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -588,7 +582,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>5</v>
@@ -605,7 +599,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>34</v>
@@ -624,12 +618,8 @@
       <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>38</v>
-      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
@@ -642,10 +632,10 @@
         <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
@@ -777,13 +767,13 @@
         <v>4</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -996,10 +986,10 @@
         <v>26</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1152,7 +1142,7 @@
         <v>4</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
feat: Support default attribution and email in attribution
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution_par_mot.xlsx
+++ b/tests/integration/test_data/test_attribution_par_mot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEE86BA-1668-5848-ACCE-3498FEEC95F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23ECE159-BED3-E446-8F1D-E6C0BE0AAB2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34400" yWindow="500" windowWidth="34400" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mots clés" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="42">
   <si>
     <t>Lecture</t>
   </si>
@@ -40,12 +40,6 @@
   </si>
   <si>
     <t>an 16</t>
-  </si>
-  <si>
-    <t>julien.dauce@sante.gouv.fr,marie.faugeron@sante.gouv.fr,marin.guedo-guilloteau@sante.gouv.fr,nathan.soto@sante.gouv.fr</t>
-  </si>
-  <si>
-    <t>Julien Dauce,Marie Faugeron,Marin Guédo-Guilloteau,Nathan Soto</t>
   </si>
   <si>
     <t>I. – À la fin du III de l’article 18 de la loi n° 2022‑1616 du 23 décembre 2022 de financement de la sécurité sociale pour 2023, le montant : « 2,21 milliards d’euros » est remplacé par le montant : « 2,35 milliards d’euros ».
@@ -95,12 +89,6 @@
     <t>I. – Le 1° du III de l’article L. 136-8 du code de la sécurité sociale est complété par un f ainsi rédigé :
   « f) L’allocation en faveur des lycéens de la voie professionnelle dans le cadre de la valorisation des périodes de formation en milieu professionnel. ».
   II. – La perte de recettes pour les organismes de sécurité sociale est compensée à due concurrence par la majoration de l’accise sur les tabacs prévue au chapitre IV du titre Ier du livre III du code des impositions sur les biens et services.</t>
-  </si>
-  <si>
-    <t>julien.dauce@sante.gouv.fr,marie.faugeron@sante.gouv.fr</t>
-  </si>
-  <si>
-    <t>Julien Dauce,Marie Faugeron</t>
   </si>
   <si>
     <t>À l’alinéa 13, substituer aux mots :
@@ -179,12 +167,6 @@
 Cette faculté est ouverte du 1er avril au 31 décembre 2023. Elle est applicable à compter de l’exercice suivant. L’exercice de cette option présente le même caractère définitif que celui prévu à l’article L. 241-18-1 du code de la sécurité sociale.</t>
   </si>
   <si>
-    <t>julien.dauce@sante.gouv.fr,marin.guedo-guilloteau@sante.gouv.fr</t>
-  </si>
-  <si>
-    <t>Julien Dauce,Marin Guédo-Guilloteau</t>
-  </si>
-  <si>
     <t>Le code général des impôts est ainsi modifié :
 1° L’article L. 1635 bis est ainsi rétabli :
 « Art. L. 1635 bis – Les usagers du système de santé bénéficient de la permanence des soins dans les conditions prévues par le présent code.</t>
@@ -240,12 +222,18 @@
   <si>
     <t>Mister Fake</t>
   </si>
+  <si>
+    <t>Etienne Barraud</t>
+  </si>
+  <si>
+    <t>etienne.barraud@sante.gouv.fr</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +258,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -302,10 +304,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -331,8 +334,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -557,9 +564,9 @@
     <col min="5" max="5" width="39.6640625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -574,7 +581,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>273</v>
       </c>
@@ -582,16 +589,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>274</v>
       </c>
@@ -599,16 +606,16 @@
         <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>720</v>
       </c>
@@ -616,12 +623,16 @@
         <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>1573</v>
       </c>
@@ -629,16 +640,16 @@
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="E5" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>1650</v>
       </c>
@@ -646,16 +657,16 @@
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>2694</v>
       </c>
@@ -663,13 +674,13 @@
         <v>4</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>14</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -691,7 +702,7 @@
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>2839</v>
       </c>
@@ -699,10 +710,14 @@
         <v>4</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="7"/>
+        <v>13</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>40</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -723,7 +738,7 @@
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>2862</v>
       </c>
@@ -731,13 +746,13 @@
         <v>4</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -759,7 +774,7 @@
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>2863</v>
       </c>
@@ -767,13 +782,13 @@
         <v>4</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -795,7 +810,7 @@
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>2959</v>
       </c>
@@ -803,13 +818,13 @@
         <v>4</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -831,7 +846,7 @@
       <c r="W11" s="2"/>
       <c r="X11" s="2"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>2967</v>
       </c>
@@ -839,13 +854,13 @@
         <v>4</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -867,7 +882,7 @@
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>2971</v>
       </c>
@@ -875,13 +890,13 @@
         <v>4</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -903,7 +918,7 @@
       <c r="W13" s="2"/>
       <c r="X13" s="2"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>2983</v>
       </c>
@@ -911,13 +926,13 @@
         <v>4</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -939,7 +954,7 @@
       <c r="W14" s="2"/>
       <c r="X14" s="2"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>3286</v>
       </c>
@@ -947,17 +962,15 @@
         <v>4</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
@@ -975,7 +988,7 @@
       <c r="W15" s="2"/>
       <c r="X15" s="2"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>3297</v>
       </c>
@@ -983,13 +996,13 @@
         <v>4</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1011,7 +1024,7 @@
       <c r="W16" s="2"/>
       <c r="X16" s="2"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>3299</v>
       </c>
@@ -1019,13 +1032,13 @@
         <v>4</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1047,7 +1060,7 @@
       <c r="W17" s="2"/>
       <c r="X17" s="2"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>3321</v>
       </c>
@@ -1055,13 +1068,13 @@
         <v>4</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1083,7 +1096,7 @@
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>3323</v>
       </c>
@@ -1091,16 +1104,16 @@
         <v>4</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>3324</v>
       </c>
@@ -1108,16 +1121,16 @@
         <v>4</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4">
         <v>3328</v>
       </c>
@@ -1125,16 +1138,16 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>3330</v>
       </c>
@@ -1142,16 +1155,16 @@
         <v>4</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>3331</v>
       </c>
@@ -1159,16 +1172,16 @@
         <v>4</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>3334</v>
       </c>
@@ -1176,16 +1189,16 @@
         <v>4</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>3335</v>
       </c>
@@ -1193,13 +1206,13 @@
         <v>4</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.2">
@@ -8031,6 +8044,11 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E1000">
     <sortCondition ref="A1:A1000"/>
   </sortState>
+  <hyperlinks>
+    <hyperlink ref="D9" r:id="rId1" xr:uid="{9BEBDAEF-ED18-9D4F-91FB-07D563D63CCF}"/>
+    <hyperlink ref="D8" r:id="rId2" display="mailto:etienne.barraud@sante.gouv.fr" xr:uid="{2A54DD46-170A-C541-9AE7-A8079584BA42}"/>
+    <hyperlink ref="D4" r:id="rId3" display="mailto:etienne.barraud@sante.gouv.fr" xr:uid="{7ABAAC0D-B7B7-3C41-BA58-B93321951BED}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
tests: Fix integration tests following some recent attribution algo changes
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_attribution_par_mot.xlsx
+++ b/tests/integration/test_data/test_attribution_par_mot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/amendements-intelligents/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23ECE159-BED3-E446-8F1D-E6C0BE0AAB2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC18F88E-E463-A442-9064-4C9959288B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mots clés" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="44">
   <si>
     <t>Lecture</t>
   </si>
@@ -227,6 +227,12 @@
   </si>
   <si>
     <t>etienne.barraud@sante.gouv.fr</t>
+  </si>
+  <si>
+    <t>nathalie.gouge@sante.gouv.fr</t>
+  </si>
+  <si>
+    <t>Nathalie Gouge</t>
   </si>
 </sst>
 </file>
@@ -659,11 +665,11 @@
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>9</v>
+      <c r="D6" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -713,10 +719,10 @@
         <v>13</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -8046,8 +8052,8 @@
   </sortState>
   <hyperlinks>
     <hyperlink ref="D9" r:id="rId1" xr:uid="{9BEBDAEF-ED18-9D4F-91FB-07D563D63CCF}"/>
-    <hyperlink ref="D8" r:id="rId2" display="mailto:etienne.barraud@sante.gouv.fr" xr:uid="{2A54DD46-170A-C541-9AE7-A8079584BA42}"/>
-    <hyperlink ref="D4" r:id="rId3" display="mailto:etienne.barraud@sante.gouv.fr" xr:uid="{7ABAAC0D-B7B7-3C41-BA58-B93321951BED}"/>
+    <hyperlink ref="D4" r:id="rId2" display="mailto:etienne.barraud@sante.gouv.fr" xr:uid="{7ABAAC0D-B7B7-3C41-BA58-B93321951BED}"/>
+    <hyperlink ref="D6" r:id="rId3" display="mailto:etienne.barraud@sante.gouv.fr" xr:uid="{03CF2FBB-CDA3-7A46-B441-8E69A3FED4CF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>